<commit_message>
feat(pro-ciclo-5): aggiornamento esercizi A25, A27, A29, Dumbbell biker squat ID 82 e progressione Salto alfiere
</commit_message>
<xml_diff>
--- a/PRO database esercizi.xlsx
+++ b/PRO database esercizi.xlsx
@@ -36158,7 +36158,7 @@
       </c>
       <c r="G212" s="3" t="inlineStr">
         <is>
-          <t>3x8+8</t>
+          <t>3x40"+40"</t>
         </is>
       </c>
       <c r="H212" s="3" t="inlineStr"/>
@@ -36199,32 +36199,28 @@
         </is>
       </c>
       <c r="E213" s="3" t="n">
-        <v>42</v>
+        <v>82</v>
       </c>
       <c r="F213" s="3" t="inlineStr">
         <is>
-          <t>Push the wall squat</t>
+          <t>Dumbbell biker's squat</t>
         </is>
       </c>
       <c r="G213" s="3" t="inlineStr">
         <is>
-          <t>3x8</t>
-        </is>
-      </c>
-      <c r="H213" s="3" t="inlineStr">
-        <is>
-          <t>45"</t>
-        </is>
-      </c>
+          <t>3x12</t>
+        </is>
+      </c>
+      <c r="H213" s="3" t="inlineStr"/>
       <c r="I213" s="3" t="inlineStr"/>
       <c r="J213" s="3" t="inlineStr">
         <is>
-          <t>jump set</t>
+          <t>jump set | usare un manubrio di peso adeguato al riscaldamento</t>
         </is>
       </c>
       <c r="K213" s="3" t="inlineStr">
         <is>
-          <t>https://youtube.com/shorts/3a_ww0jGYsM</t>
+          <t>https://youtu.be/jqhow36DTdg</t>
         </is>
       </c>
       <c r="L213" s="3" t="inlineStr"/>
@@ -36262,7 +36258,7 @@
       </c>
       <c r="G214" s="3" t="inlineStr">
         <is>
-          <t>4x5+5</t>
+          <t>4x10</t>
         </is>
       </c>
       <c r="H214" s="3" t="inlineStr">
@@ -36273,7 +36269,7 @@
       <c r="I214" s="3" t="inlineStr"/>
       <c r="J214" s="3" t="inlineStr">
         <is>
-          <t>RPE 8.5</t>
+          <t>RPE 8.5 | fare un corretto avvicinamento</t>
         </is>
       </c>
       <c r="K214" s="3" t="inlineStr">
@@ -36407,7 +36403,7 @@
       </c>
       <c r="D217" s="3" t="inlineStr">
         <is>
-          <t>4a</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E217" s="3" t="n">
@@ -36420,14 +36416,14 @@
       </c>
       <c r="G217" s="3" t="inlineStr">
         <is>
-          <t>3x6+6</t>
+          <t>studio progressivo 5-10 minuti</t>
         </is>
       </c>
       <c r="H217" s="3" t="inlineStr"/>
       <c r="I217" s="3" t="inlineStr"/>
       <c r="J217" s="3" t="inlineStr">
         <is>
-          <t>circuito (3 round)</t>
+          <t>Dal momento che è un esercizio di impatto e affrontato per la prima volta, viene richiesto un lavoro preventivo di studio progressivo fino a realizzare il movimento intero e proseguito.</t>
         </is>
       </c>
       <c r="K217" s="3" t="inlineStr">
@@ -36457,7 +36453,7 @@
       </c>
       <c r="D218" s="3" t="inlineStr">
         <is>
-          <t>4b</t>
+          <t>5a</t>
         </is>
       </c>
       <c r="E218" s="3" t="n">
@@ -36477,7 +36473,7 @@
       <c r="I218" s="3" t="inlineStr"/>
       <c r="J218" s="3" t="inlineStr">
         <is>
-          <t>circuito (3 round)</t>
+          <t>jump set</t>
         </is>
       </c>
       <c r="K218" s="3" t="inlineStr"/>
@@ -36503,7 +36499,7 @@
       </c>
       <c r="D219" s="3" t="inlineStr">
         <is>
-          <t>4c</t>
+          <t>5b</t>
         </is>
       </c>
       <c r="E219" s="3" t="n">
@@ -36527,7 +36523,7 @@
       <c r="I219" s="3" t="inlineStr"/>
       <c r="J219" s="3" t="inlineStr">
         <is>
-          <t>circuito (3 round)</t>
+          <t>jump set</t>
         </is>
       </c>
       <c r="K219" s="3" t="inlineStr">
@@ -37028,7 +37024,7 @@
       </c>
       <c r="G229" s="3" t="inlineStr">
         <is>
-          <t>3x8+8</t>
+          <t>3x40"+40"</t>
         </is>
       </c>
       <c r="H229" s="3" t="inlineStr"/>
@@ -37069,32 +37065,28 @@
         </is>
       </c>
       <c r="E230" s="3" t="n">
-        <v>42</v>
+        <v>82</v>
       </c>
       <c r="F230" s="3" t="inlineStr">
         <is>
-          <t>Push the wall squat</t>
+          <t>Dumbbell biker's squat</t>
         </is>
       </c>
       <c r="G230" s="3" t="inlineStr">
         <is>
-          <t>3x8</t>
-        </is>
-      </c>
-      <c r="H230" s="3" t="inlineStr">
-        <is>
-          <t>45"</t>
-        </is>
-      </c>
+          <t>3x12</t>
+        </is>
+      </c>
+      <c r="H230" s="3" t="inlineStr"/>
       <c r="I230" s="3" t="inlineStr"/>
       <c r="J230" s="3" t="inlineStr">
         <is>
-          <t>jump set</t>
+          <t>jump set | usare un manubrio di peso adeguato al riscaldamento</t>
         </is>
       </c>
       <c r="K230" s="3" t="inlineStr">
         <is>
-          <t>https://youtube.com/shorts/3a_ww0jGYsM</t>
+          <t>https://youtu.be/jqhow36DTdg</t>
         </is>
       </c>
       <c r="L230" s="3" t="inlineStr"/>
@@ -37132,7 +37124,7 @@
       </c>
       <c r="G231" s="3" t="inlineStr">
         <is>
-          <t>4x5+5</t>
+          <t>4x10</t>
         </is>
       </c>
       <c r="H231" s="3" t="inlineStr">
@@ -37143,7 +37135,7 @@
       <c r="I231" s="3" t="inlineStr"/>
       <c r="J231" s="3" t="inlineStr">
         <is>
-          <t>RPE 8.5</t>
+          <t>RPE 8.5 | fare un corretto avvicinamento</t>
         </is>
       </c>
       <c r="K231" s="3" t="inlineStr">
@@ -37290,14 +37282,14 @@
       </c>
       <c r="G234" s="3" t="inlineStr">
         <is>
-          <t>3x6+6</t>
+          <t>3x5+5</t>
         </is>
       </c>
       <c r="H234" s="3" t="inlineStr"/>
       <c r="I234" s="3" t="inlineStr"/>
       <c r="J234" s="3" t="inlineStr">
         <is>
-          <t>circuito (3 round)</t>
+          <t>jump set</t>
         </is>
       </c>
       <c r="K234" s="3" t="inlineStr">
@@ -37331,26 +37323,34 @@
         </is>
       </c>
       <c r="E235" s="3" t="n">
-        <v>96</v>
+        <v>3</v>
       </c>
       <c r="F235" s="3" t="inlineStr">
         <is>
-          <t>coiled Ax Sit up</t>
+          <t>skierg pagaia alternato</t>
         </is>
       </c>
       <c r="G235" s="3" t="inlineStr">
         <is>
-          <t>3x8+8</t>
-        </is>
-      </c>
-      <c r="H235" s="3" t="inlineStr"/>
+          <t>3x30"+30"</t>
+        </is>
+      </c>
+      <c r="H235" s="3" t="inlineStr">
+        <is>
+          <t>60"</t>
+        </is>
+      </c>
       <c r="I235" s="3" t="inlineStr"/>
       <c r="J235" s="3" t="inlineStr">
         <is>
-          <t>circuito (3 round)</t>
-        </is>
-      </c>
-      <c r="K235" s="3" t="inlineStr"/>
+          <t>jump set</t>
+        </is>
+      </c>
+      <c r="K235" s="3" t="inlineStr">
+        <is>
+          <t>https://youtube.com/shorts/7n-hAJAXoYU</t>
+        </is>
+      </c>
       <c r="L235" s="3" t="inlineStr"/>
       <c r="M235" s="2" t="n"/>
       <c r="N235" s="2" t="n"/>
@@ -37373,38 +37373,30 @@
       </c>
       <c r="D236" s="3" t="inlineStr">
         <is>
-          <t>4c</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E236" s="3" t="n">
-        <v>3</v>
+        <v>96</v>
       </c>
       <c r="F236" s="3" t="inlineStr">
         <is>
-          <t>skierg pagaia alternato</t>
+          <t>coiled Ax Sit up</t>
         </is>
       </c>
       <c r="G236" s="3" t="inlineStr">
         <is>
-          <t>3x30"+30"</t>
+          <t>3x8+8</t>
         </is>
       </c>
       <c r="H236" s="3" t="inlineStr">
         <is>
-          <t>60"</t>
+          <t>45"</t>
         </is>
       </c>
       <c r="I236" s="3" t="inlineStr"/>
-      <c r="J236" s="3" t="inlineStr">
-        <is>
-          <t>circuito (3 round)</t>
-        </is>
-      </c>
-      <c r="K236" s="3" t="inlineStr">
-        <is>
-          <t>https://youtube.com/shorts/7n-hAJAXoYU</t>
-        </is>
-      </c>
+      <c r="J236" s="3" t="inlineStr"/>
+      <c r="K236" s="3" t="inlineStr"/>
       <c r="L236" s="3" t="inlineStr"/>
       <c r="M236" s="2" t="n"/>
       <c r="N236" s="2" t="n"/>
@@ -37898,7 +37890,7 @@
       </c>
       <c r="G246" s="3" t="inlineStr">
         <is>
-          <t>3x8+8</t>
+          <t>3x40"+40"</t>
         </is>
       </c>
       <c r="H246" s="3" t="inlineStr"/>
@@ -37939,32 +37931,28 @@
         </is>
       </c>
       <c r="E247" s="3" t="n">
-        <v>42</v>
+        <v>82</v>
       </c>
       <c r="F247" s="3" t="inlineStr">
         <is>
-          <t>Push the wall squat</t>
+          <t>Dumbbell biker's squat</t>
         </is>
       </c>
       <c r="G247" s="3" t="inlineStr">
         <is>
-          <t>3x8</t>
-        </is>
-      </c>
-      <c r="H247" s="3" t="inlineStr">
-        <is>
-          <t>45"</t>
-        </is>
-      </c>
+          <t>3x12</t>
+        </is>
+      </c>
+      <c r="H247" s="3" t="inlineStr"/>
       <c r="I247" s="3" t="inlineStr"/>
       <c r="J247" s="3" t="inlineStr">
         <is>
-          <t>jump set</t>
+          <t>jump set | usare un manubrio di peso adeguato al riscaldamento</t>
         </is>
       </c>
       <c r="K247" s="3" t="inlineStr">
         <is>
-          <t>https://youtube.com/shorts/3a_ww0jGYsM</t>
+          <t>https://youtu.be/jqhow36DTdg</t>
         </is>
       </c>
       <c r="L247" s="3" t="inlineStr"/>
@@ -38002,7 +37990,7 @@
       </c>
       <c r="G248" s="3" t="inlineStr">
         <is>
-          <t>4x5+5</t>
+          <t>4x10</t>
         </is>
       </c>
       <c r="H248" s="3" t="inlineStr">
@@ -38013,7 +38001,7 @@
       <c r="I248" s="3" t="inlineStr"/>
       <c r="J248" s="3" t="inlineStr">
         <is>
-          <t>RPE 8.5</t>
+          <t>RPE 8.5 | fare un corretto avvicinamento</t>
         </is>
       </c>
       <c r="K248" s="3" t="inlineStr">
@@ -38160,7 +38148,7 @@
       </c>
       <c r="G251" s="3" t="inlineStr">
         <is>
-          <t>3x6+6</t>
+          <t>3x5+5</t>
         </is>
       </c>
       <c r="H251" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
feat(fisco-allenamenti): persistenza e sync versamenti SGG, correzione nominale side kick through e parametri Ciclo 5B
</commit_message>
<xml_diff>
--- a/PRO database esercizi.xlsx
+++ b/PRO database esercizi.xlsx
@@ -7025,7 +7025,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>medball side kick thrue</t>
+          <t>medball side kick through</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -12225,7 +12225,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>medball side kick thrue</t>
+          <t>medball side kick through</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -14328,7 +14328,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>medball side kick thrue</t>
+          <t>medball side kick through</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -17074,7 +17074,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>medball side kick thrue</t>
+          <t>medball side kick through</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -20008,7 +20008,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>medball side kick thrue</t>
+          <t>medball side kick through</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -22197,7 +22197,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>medball side kick thrue</t>
+          <t>medball side kick through</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -25115,7 +25115,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>medball side kick thrue</t>
+          <t>medball side kick through</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -36923,7 +36923,7 @@
       </c>
       <c r="F227" s="4" t="inlineStr">
         <is>
-          <t>medball side kick thrue</t>
+          <t>medball side kick through</t>
         </is>
       </c>
       <c r="G227" s="4" t="inlineStr">
@@ -37789,7 +37789,7 @@
       </c>
       <c r="F244" s="4" t="inlineStr">
         <is>
-          <t>medball side kick thrue</t>
+          <t>medball side kick through</t>
         </is>
       </c>
       <c r="G244" s="4" t="inlineStr">
@@ -38655,7 +38655,7 @@
       </c>
       <c r="F261" s="4" t="inlineStr">
         <is>
-          <t>medball side kick thrue</t>
+          <t>medball side kick through</t>
         </is>
       </c>
       <c r="G261" s="4" t="inlineStr">

</xml_diff>

<commit_message>
feat(ciclo-5): aggiornamento parametri Biker's Squat e Salto Alfiere per allenamenti 25, 27 e 29
</commit_message>
<xml_diff>
--- a/PRO database esercizi.xlsx
+++ b/PRO database esercizi.xlsx
@@ -36208,7 +36208,7 @@
       </c>
       <c r="G213" s="3" t="inlineStr">
         <is>
-          <t>3x12</t>
+          <t>3 X 12+12</t>
         </is>
       </c>
       <c r="H213" s="3" t="inlineStr"/>
@@ -36416,7 +36416,7 @@
       </c>
       <c r="G217" s="3" t="inlineStr">
         <is>
-          <t>studio progressivo 5-10 minuti</t>
+          <t>3 X 60"</t>
         </is>
       </c>
       <c r="H217" s="3" t="inlineStr"/>
@@ -36557,16 +36557,16 @@
         </is>
       </c>
       <c r="E220" s="4" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F220" s="4" t="inlineStr">
         <is>
-          <t>Cat-cow</t>
+          <t>Ground Stretch</t>
         </is>
       </c>
       <c r="G220" s="4" t="inlineStr">
         <is>
-          <t>3x12</t>
+          <t>3x10+10</t>
         </is>
       </c>
       <c r="H220" s="4" t="inlineStr"/>
@@ -36576,11 +36576,7 @@
           <t>jump set</t>
         </is>
       </c>
-      <c r="K220" s="4" t="inlineStr">
-        <is>
-          <t>https://youtube.com/shorts/EBQD1Sha26k?si=VlMRufJ_KWHm-_V1</t>
-        </is>
-      </c>
+      <c r="K220" s="4" t="inlineStr"/>
       <c r="L220" s="4" t="inlineStr"/>
       <c r="M220" s="2" t="n"/>
       <c r="N220" s="2" t="n"/>
@@ -36675,7 +36671,7 @@
       </c>
       <c r="H222" s="4" t="inlineStr">
         <is>
-          <t>RBS 60"</t>
+          <t>Rec 60"</t>
         </is>
       </c>
       <c r="I222" s="4" t="inlineStr"/>
@@ -36724,12 +36720,12 @@
       </c>
       <c r="G223" s="4" t="inlineStr">
         <is>
-          <t>4x6+6</t>
+          <t>4x12</t>
         </is>
       </c>
       <c r="H223" s="4" t="inlineStr">
         <is>
-          <t>RBS 60"</t>
+          <t>Rec 60"</t>
         </is>
       </c>
       <c r="I223" s="4" t="inlineStr"/>
@@ -36778,7 +36774,7 @@
       </c>
       <c r="G224" s="4" t="inlineStr">
         <is>
-          <t>4x30"+30"</t>
+          <t>4x40"+40"</t>
         </is>
       </c>
       <c r="H224" s="4" t="inlineStr"/>
@@ -36928,7 +36924,7 @@
       </c>
       <c r="G227" s="4" t="inlineStr">
         <is>
-          <t>x 8</t>
+          <t>x 8+8</t>
         </is>
       </c>
       <c r="H227" s="4" t="inlineStr"/>
@@ -37074,14 +37070,14 @@
       </c>
       <c r="G230" s="3" t="inlineStr">
         <is>
-          <t>3x12</t>
+          <t>3 X 12</t>
         </is>
       </c>
       <c r="H230" s="3" t="inlineStr"/>
       <c r="I230" s="3" t="inlineStr"/>
       <c r="J230" s="3" t="inlineStr">
         <is>
-          <t>jump set | usare un manubrio di peso adeguato al riscaldamento</t>
+          <t>jump set | usare un manubrio di peso adeguato al riscaldamento (alternato)</t>
         </is>
       </c>
       <c r="K230" s="3" t="inlineStr">
@@ -37282,7 +37278,7 @@
       </c>
       <c r="G234" s="3" t="inlineStr">
         <is>
-          <t>3x5+5</t>
+          <t>3 X 50"</t>
         </is>
       </c>
       <c r="H234" s="3" t="inlineStr"/>
@@ -37423,16 +37419,16 @@
         </is>
       </c>
       <c r="E237" s="4" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F237" s="4" t="inlineStr">
         <is>
-          <t>Cat-cow</t>
+          <t>Ground Stretch</t>
         </is>
       </c>
       <c r="G237" s="4" t="inlineStr">
         <is>
-          <t>3x12</t>
+          <t>3x10+10</t>
         </is>
       </c>
       <c r="H237" s="4" t="inlineStr"/>
@@ -37442,11 +37438,7 @@
           <t>jump set</t>
         </is>
       </c>
-      <c r="K237" s="4" t="inlineStr">
-        <is>
-          <t>https://youtube.com/shorts/EBQD1Sha26k?si=VlMRufJ_KWHm-_V1</t>
-        </is>
-      </c>
+      <c r="K237" s="4" t="inlineStr"/>
       <c r="L237" s="4" t="inlineStr"/>
       <c r="M237" s="2" t="n"/>
       <c r="N237" s="2" t="n"/>
@@ -37541,7 +37533,7 @@
       </c>
       <c r="H239" s="4" t="inlineStr">
         <is>
-          <t>RBS 60"</t>
+          <t>Rec 60"</t>
         </is>
       </c>
       <c r="I239" s="4" t="inlineStr"/>
@@ -37590,12 +37582,12 @@
       </c>
       <c r="G240" s="4" t="inlineStr">
         <is>
-          <t>4x6+6</t>
+          <t>4x12</t>
         </is>
       </c>
       <c r="H240" s="4" t="inlineStr">
         <is>
-          <t>RBS 60"</t>
+          <t>Rec 60"</t>
         </is>
       </c>
       <c r="I240" s="4" t="inlineStr"/>
@@ -37644,7 +37636,7 @@
       </c>
       <c r="G241" s="4" t="inlineStr">
         <is>
-          <t>4x30"+30"</t>
+          <t>4x40"+40"</t>
         </is>
       </c>
       <c r="H241" s="4" t="inlineStr"/>
@@ -37794,7 +37786,7 @@
       </c>
       <c r="G244" s="4" t="inlineStr">
         <is>
-          <t>x 8</t>
+          <t>x 8+8</t>
         </is>
       </c>
       <c r="H244" s="4" t="inlineStr"/>
@@ -37940,14 +37932,14 @@
       </c>
       <c r="G247" s="3" t="inlineStr">
         <is>
-          <t>3x12</t>
+          <t>3 X 12</t>
         </is>
       </c>
       <c r="H247" s="3" t="inlineStr"/>
       <c r="I247" s="3" t="inlineStr"/>
       <c r="J247" s="3" t="inlineStr">
         <is>
-          <t>jump set | usare un manubrio di peso adeguato al riscaldamento</t>
+          <t>jump set | usare un manubrio di peso adeguato al riscaldamento (alternato)</t>
         </is>
       </c>
       <c r="K247" s="3" t="inlineStr">
@@ -38148,7 +38140,7 @@
       </c>
       <c r="G251" s="3" t="inlineStr">
         <is>
-          <t>3x5+5</t>
+          <t>3 X 45"</t>
         </is>
       </c>
       <c r="H251" s="3" t="inlineStr"/>
@@ -38289,16 +38281,16 @@
         </is>
       </c>
       <c r="E254" s="4" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F254" s="4" t="inlineStr">
         <is>
-          <t>Cat-cow</t>
+          <t>Ground Stretch</t>
         </is>
       </c>
       <c r="G254" s="4" t="inlineStr">
         <is>
-          <t>3x12</t>
+          <t>3x10+10</t>
         </is>
       </c>
       <c r="H254" s="4" t="inlineStr"/>
@@ -38308,11 +38300,7 @@
           <t>jump set</t>
         </is>
       </c>
-      <c r="K254" s="4" t="inlineStr">
-        <is>
-          <t>https://youtube.com/shorts/EBQD1Sha26k?si=VlMRufJ_KWHm-_V1</t>
-        </is>
-      </c>
+      <c r="K254" s="4" t="inlineStr"/>
       <c r="L254" s="4" t="inlineStr"/>
       <c r="M254" s="2" t="n"/>
       <c r="N254" s="2" t="n"/>
@@ -38407,7 +38395,7 @@
       </c>
       <c r="H256" s="4" t="inlineStr">
         <is>
-          <t>RBS 60"</t>
+          <t>Rec 60"</t>
         </is>
       </c>
       <c r="I256" s="4" t="inlineStr"/>
@@ -38456,12 +38444,12 @@
       </c>
       <c r="G257" s="4" t="inlineStr">
         <is>
-          <t>4x6+6</t>
+          <t>4x12</t>
         </is>
       </c>
       <c r="H257" s="4" t="inlineStr">
         <is>
-          <t>RBS 60"</t>
+          <t>Rec 60"</t>
         </is>
       </c>
       <c r="I257" s="4" t="inlineStr"/>
@@ -38510,7 +38498,7 @@
       </c>
       <c r="G258" s="4" t="inlineStr">
         <is>
-          <t>4x30"+30"</t>
+          <t>4x40"+40"</t>
         </is>
       </c>
       <c r="H258" s="4" t="inlineStr"/>
@@ -38660,7 +38648,7 @@
       </c>
       <c r="G261" s="4" t="inlineStr">
         <is>
-          <t>x 8</t>
+          <t>x 8+8</t>
         </is>
       </c>
       <c r="H261" s="4" t="inlineStr"/>

</xml_diff>